<commit_message>
Add NPV formula sheet to Week 7 valuation workbook
</commit_message>
<xml_diff>
--- a/weeks/week-07/local-business-valuation-activity.xlsx
+++ b/weeks/week-07/local-business-valuation-activity.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Activity" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPV Formula" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1208,4 +1209,253 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>NPV Formula Version</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>This sheet uses Excel's NPV function directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NPV formula used: =NPV(discount_rate, year_1:year_5_cash_flows)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Investment value formula used: =NPV(discount_rate, cash_flows) - asking_price</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Discount Rate</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Asking Price</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>NPV of Cash Flows</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>NPV Minus Asking Price</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Elsah Coffee Cart</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>92000</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>22000</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>26000</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>27000</v>
+      </c>
+      <c r="I7" s="10">
+        <f>NPV(B7,D7:H7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="10">
+        <f>I7-C7</f>
+        <v/>
+      </c>
+      <c r="K7" s="9">
+        <f>IF(J7&gt;0,"Looks undervalued","Looks overvalued")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Riverbend HVAC Service</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>165000</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>38000</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>44000</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>52000</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>60000</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>68000</v>
+      </c>
+      <c r="I8" s="10">
+        <f>NPV(B8,D8:H8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="10">
+        <f>I8-C8</f>
+        <v/>
+      </c>
+      <c r="K8" s="9">
+        <f>IF(J8&gt;0,"Looks undervalued","Looks overvalued")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Campus Gear Rental App</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>34000</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>75000</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>130000</v>
+      </c>
+      <c r="I9" s="10">
+        <f>NPV(B9,D9:H9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="10">
+        <f>I9-C9</f>
+        <v/>
+      </c>
+      <c r="K9" s="9">
+        <f>IF(J9&gt;0,"Looks undervalued","Looks overvalued")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Student Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>How does this NPV formula sheet compare to the present-value-by-year sheet?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:K13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>